<commit_message>
tc 8 - 13 OK
</commit_message>
<xml_diff>
--- a/Casos.xlsx
+++ b/Casos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\Desktop\SOFT311\PROYECTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18EE0E3-87FB-4E8C-9F5B-62CEAADAE374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C80BFCC-DB42-4AFC-8BEE-2BE7550F44AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-001 Sign Up" sheetId="25" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="96">
   <si>
     <t>Pasos</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Login</t>
   </si>
   <si>
-    <t xml:space="preserve">Validación de formato email en suscripción </t>
-  </si>
-  <si>
     <t>Ingreso a la pantalla de productos por medio del botón Shop Now</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
   </si>
   <si>
     <t>TC-006</t>
-  </si>
-  <si>
-    <t>Cart</t>
   </si>
   <si>
     <t>TC-007</t>
@@ -284,9 +278,6 @@
 6. Dar click en botón Send Message</t>
   </si>
   <si>
-    <t>Exitoso, el mensaje se envía correctamente</t>
-  </si>
-  <si>
     <t>Ir a la página https://storedemo.testdino.com</t>
   </si>
   <si>
@@ -303,17 +294,7 @@
     <t>Exitoso, si se redirecciona a la página de los productos, sin embargo no se marca la opción del menú superior correctamente</t>
   </si>
   <si>
-    <t>Validar cantidad del elementos agregados a favoritos con éxito, desde página All products</t>
-  </si>
-  <si>
     <t>Ir a la página https://storedemo.testdino.com/products</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.  Estar en la pagina https://storedemo.testdino.com/products
-2.  Agregar productos a favoritos dando click en el botón de corazón
-3.  Validar la cantidad de productos agregados a favoritos (en la esquina derecha arriba en el ícono de corazón)
-4. 
-5. </t>
   </si>
   <si>
     <t>Exitoso, se muestra correctamente la cantidad de favoritos</t>
@@ -351,19 +332,6 @@
     <t>Ir a la página https://storedemo.testdino.com/</t>
   </si>
   <si>
-    <t>Your Email: 12345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Estar en la página https://storedemo.testdino.com en la sección Suscribe
-2.  Ingresar Your Email: 12345
-3.  Dar click en botón Suscribe
-4.  Validar que no lo deje suscribir 
-5. </t>
-  </si>
-  <si>
-    <t>Exitoso, se espera que no permita que se suscriba, pero si lo permite</t>
-  </si>
-  <si>
     <t>First Name: Nayeli
 Last Name: Castillo
 Subject: consulta
@@ -401,6 +369,45 @@
   </si>
   <si>
     <t>Exitoso, muestra el mensaje correctamente</t>
+  </si>
+  <si>
+    <t>First Name: Nayeli
+Last Name: Castillo
+Subject: consulta 
+Your Message: Hola, me pueden brindar el número de télefono, por favor.</t>
+  </si>
+  <si>
+    <t>Exitoso, el mensaje se envía correctamente y muestra un mesaje de éxito</t>
+  </si>
+  <si>
+    <t>Cart - Home</t>
+  </si>
+  <si>
+    <t>Validar remover favorito desde pagina de wishlist</t>
+  </si>
+  <si>
+    <t>1.  Estar en la pagina https://storedemo.testdino.com/products
+2.  Agregar productos a favoritos dando click en el botón de corazón
+3.  Dar click en el icono de corazon para redirigirse a la pantalla https://storedemo.testdino.com/wishlist
+4. Validar que se este en la pantalla de wishlist
+5. Dar click en el icono de borrar de un card de producto
+6. Validar que se remueve el producto por medio del mensaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validación de suscripción </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Estar en la página https://storedemo.testdino.com en la sección Suscribe
+2.  Ingresar Your Email: naye2@test.com
+3.  Dar click en botón Suscribe
+4.  Validar que se suscriba el email 
+5. </t>
+  </si>
+  <si>
+    <t>Exitoso, se suscribio correctamente</t>
+  </si>
+  <si>
+    <t>Your Email: naye2@test.com</t>
   </si>
 </sst>
 </file>
@@ -842,7 +849,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -850,7 +857,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -864,7 +871,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -872,7 +879,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -880,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -888,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -927,7 +934,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -935,7 +942,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -943,7 +950,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -957,7 +964,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -965,7 +972,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -973,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -981,7 +988,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -989,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1020,7 +1027,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1028,7 +1035,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1036,7 +1043,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1050,7 +1057,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1058,7 +1065,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1066,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1074,7 +1081,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1082,7 +1089,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1113,7 +1120,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1121,7 +1128,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1129,7 +1136,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1143,7 +1150,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1157,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1165,7 +1172,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1204,7 +1211,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1212,7 +1219,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1220,7 +1227,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1234,7 +1241,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1248,7 +1255,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1256,7 +1263,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1295,7 +1302,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1311,7 +1318,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1325,7 +1332,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1333,7 +1340,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1341,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1349,7 +1356,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1357,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1365,7 +1372,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1388,7 +1395,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1396,7 +1403,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1404,7 +1411,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1418,7 +1425,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1432,7 +1439,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1440,7 +1447,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1448,7 +1455,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1479,7 +1486,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1487,7 +1494,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1495,7 +1502,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1509,7 +1516,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1523,7 +1530,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1531,7 +1538,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1539,7 +1546,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1547,7 +1554,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1570,7 +1577,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1578,7 +1585,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1586,7 +1593,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1600,7 +1607,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1614,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1622,7 +1629,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1630,7 +1637,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1661,7 +1668,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1669,7 +1676,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1677,7 +1684,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1691,21 +1698,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1713,7 +1722,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1752,7 +1761,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1760,7 +1769,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1768,7 +1777,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1782,7 +1791,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1796,7 +1805,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1804,7 +1813,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1812,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1835,7 +1844,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="86.85546875" customWidth="1"/>
+    <col min="2" max="2" width="96.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1843,7 +1852,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1851,7 +1860,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1859,7 +1868,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1873,7 +1882,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1882,12 +1891,12 @@
       </c>
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1895,7 +1904,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1903,7 +1912,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1934,7 +1943,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1950,7 +1959,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1964,7 +1973,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1972,7 +1981,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1980,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1988,7 +1997,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1996,7 +2005,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>